<commit_message>
Align delivery to copy link; add blank versions and buyer guide PDF
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/seller-profit-tracker/dist/MarginKite-Etsy-Fee-Calculator-Lite.xlsx
+++ b/products/seller-profit-tracker/dist/MarginKite-Etsy-Fee-Calculator-Lite.xlsx
@@ -147,6 +147,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="00DDEBF7"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -508,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F35"/>
+  <dimension ref="B1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -941,12 +948,52 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Google Sheets: sign in to Google, open the "make a copy" link from your download page, then click Make a copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Excel: open the .xlsx in Excel 2016 or newer. There are no macros to allow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>No link handy? Upload the .xlsx to Google Drive, then choose File &gt; Save as Google Sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Two versions: MarginKite-Etsy-Fee-Calculator-Lite.xlsx has an example item; MarginKite-Etsy-Fee-Calculator-Lite-BLANK.xlsx starts empty. This is the example version.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B24:E24"/>
   </mergeCells>
+  <conditionalFormatting sqref="C13:C21">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>$C$5=""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="C9 C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Pick from the list" error="Please pick a value from the list." type="list">
       <formula1>"Y,N"</formula1>

</xml_diff>